<commit_message>
Buch und Story 10
</commit_message>
<xml_diff>
--- a/docs/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/docs/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF3AA2E-AB77-44A1-83E5-0736D56546DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4F376F-FFD5-4C39-916C-B98CE95F47AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="193">
   <si>
     <t>Höllisch</t>
   </si>
@@ -601,6 +601,9 @@
   </si>
   <si>
     <t>Destruction and Pain</t>
+  </si>
+  <si>
+    <t>Die Sprache der Hölle wird auf die Haut von Höllenbrut geschrieben mit Strähnen aus einem Metall asu der Hölle, welches es nur dort gibt.</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB64"/>
+  <dimension ref="A1:AA64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -1132,7 +1135,7 @@
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>96</v>
       </c>
@@ -1145,9 +1148,10 @@
       <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -1159,9 +1163,8 @@
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>147</v>
       </c>
@@ -1171,47 +1174,47 @@
       <c r="C2" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>46</v>
       </c>
+      <c r="F2" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="G2" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1221,7 +1224,8 @@
       <c r="C3" t="s">
         <v>151</v>
       </c>
-      <c r="F3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
@@ -1232,10 +1236,9 @@
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="8"/>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="Q3" s="8"/>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -1245,47 +1248,47 @@
       <c r="C4" t="s">
         <v>152</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>53</v>
       </c>
+      <c r="F4" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="G4" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q4" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="Q4" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -1295,7 +1298,8 @@
       <c r="C5" t="s">
         <v>153</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -1306,10 +1310,9 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="10"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="Q5" s="10"/>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>99</v>
       </c>
@@ -1319,77 +1322,77 @@
       <c r="C6" t="s">
         <v>154</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>24</v>
       </c>
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="Z6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="AA6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AB6" s="5" t="s">
+      <c r="AA6" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>105</v>
       </c>
@@ -1399,14 +1402,15 @@
       <c r="C7" t="s">
         <v>155</v>
       </c>
-      <c r="F7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
@@ -1420,10 +1424,9 @@
       <c r="X7" s="7"/>
       <c r="Y7" s="7"/>
       <c r="Z7" s="7"/>
-      <c r="AA7" s="7"/>
-      <c r="AB7" s="8"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AA7" s="8"/>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>106</v>
       </c>
@@ -1433,32 +1436,32 @@
       <c r="C8" t="s">
         <v>156</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="E8" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="F8" s="17" t="s">
         <v>111</v>
       </c>
+      <c r="G8" s="12" t="s">
+        <v>112</v>
+      </c>
       <c r="H8" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="L8" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="L8" s="13" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -1468,32 +1471,32 @@
       <c r="C9" t="s">
         <v>123</v>
       </c>
-      <c r="F9" s="14">
+      <c r="E9" s="14">
         <v>0</v>
       </c>
+      <c r="F9" s="15">
+        <v>1</v>
+      </c>
       <c r="G9" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" s="15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9" s="15">
-        <v>5</v>
-      </c>
-      <c r="L9" s="15">
         <v>6</v>
       </c>
-      <c r="M9" s="16">
+      <c r="L9" s="16">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>122</v>
       </c>
@@ -1504,7 +1507,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>120</v>
       </c>
@@ -1514,11 +1517,14 @@
       <c r="C11" t="s">
         <v>158</v>
       </c>
-      <c r="F11" t="s">
+      <c r="E11" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="N11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -1528,11 +1534,11 @@
       <c r="C12" t="s">
         <v>159</v>
       </c>
-      <c r="F12" t="s">
+      <c r="E12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -1542,11 +1548,11 @@
       <c r="C13" t="s">
         <v>134</v>
       </c>
-      <c r="F13" t="s">
+      <c r="E13" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>129</v>
       </c>
@@ -1556,11 +1562,11 @@
       <c r="C14" t="s">
         <v>160</v>
       </c>
-      <c r="F14" t="s">
+      <c r="E14" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>127</v>
       </c>
@@ -1570,11 +1576,11 @@
       <c r="C15" t="s">
         <v>161</v>
       </c>
-      <c r="F15" t="s">
+      <c r="E15" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>143</v>
       </c>
@@ -1584,11 +1590,11 @@
       <c r="C16" t="s">
         <v>145</v>
       </c>
-      <c r="F16" t="s">
+      <c r="E16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>132</v>
       </c>
@@ -1598,11 +1604,11 @@
       <c r="C17" t="s">
         <v>151</v>
       </c>
-      <c r="F17" t="s">
+      <c r="E17" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>130</v>
       </c>
@@ -1612,11 +1618,11 @@
       <c r="C18" t="s">
         <v>162</v>
       </c>
-      <c r="F18" t="s">
+      <c r="E18" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>136</v>
       </c>
@@ -1627,7 +1633,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>138</v>
       </c>
@@ -1637,11 +1643,11 @@
       <c r="C20" t="s">
         <v>137</v>
       </c>
-      <c r="F20" t="s">
+      <c r="E20" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>140</v>
       </c>
@@ -1651,11 +1657,11 @@
       <c r="C21" t="s">
         <v>163</v>
       </c>
-      <c r="F21" t="s">
+      <c r="E21" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>141</v>
       </c>
@@ -1665,11 +1671,11 @@
       <c r="C22" t="s">
         <v>164</v>
       </c>
-      <c r="F22" t="s">
+      <c r="E22" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>142</v>
       </c>
@@ -1679,11 +1685,11 @@
       <c r="C23" t="s">
         <v>38</v>
       </c>
-      <c r="F23" t="s">
+      <c r="E23" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>149</v>
       </c>
@@ -1693,11 +1699,11 @@
       <c r="C24" t="s">
         <v>182</v>
       </c>
-      <c r="F24" t="s">
+      <c r="E24" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>169</v>
       </c>
@@ -1707,11 +1713,11 @@
       <c r="C25" t="s">
         <v>181</v>
       </c>
-      <c r="F25" t="s">
+      <c r="E25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>167</v>
       </c>
@@ -1721,11 +1727,11 @@
       <c r="C26" t="s">
         <v>170</v>
       </c>
-      <c r="F26" t="s">
+      <c r="E26" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>171</v>
       </c>
@@ -1735,11 +1741,11 @@
       <c r="C27" t="s">
         <v>173</v>
       </c>
-      <c r="F27" t="s">
+      <c r="E27" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>175</v>
       </c>
@@ -1749,11 +1755,11 @@
       <c r="C28" t="s">
         <v>174</v>
       </c>
-      <c r="F28" t="s">
+      <c r="E28" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>177</v>
       </c>
@@ -1763,11 +1769,11 @@
       <c r="C29" t="s">
         <v>29</v>
       </c>
-      <c r="F29" t="s">
+      <c r="E29" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>188</v>
       </c>
@@ -1777,11 +1783,11 @@
       <c r="C30" t="s">
         <v>190</v>
       </c>
-      <c r="F30" t="s">
+      <c r="E30" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>186</v>
       </c>
@@ -1791,11 +1797,11 @@
       <c r="C31" t="s">
         <v>185</v>
       </c>
-      <c r="F31" t="s">
+      <c r="E31" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>171</v>
       </c>
@@ -1805,11 +1811,11 @@
       <c r="C32" t="s">
         <v>183</v>
       </c>
-      <c r="F32" t="s">
+      <c r="E32" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>179</v>
       </c>
@@ -1819,11 +1825,11 @@
       <c r="C33" t="s">
         <v>165</v>
       </c>
-      <c r="F33" t="s">
+      <c r="E33" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>178</v>
       </c>
@@ -1834,128 +1840,128 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F35" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F36" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F38" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F39" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E39" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F41" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E41" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F42" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F43" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F44" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E44" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F45" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E45" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F46" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E46" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F48" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E48" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F49" t="s">
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F50" t="s">
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F51" t="s">
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F52" t="s">
+    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E52" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F53" t="s">
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E53" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F54" t="s">
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F55" t="s">
+    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E55" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F56" t="s">
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E56" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F57" t="s">
+    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E57" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F58" t="s">
+    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E58" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F60" t="s">
+    <row r="60" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E60" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="61" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F61" t="s">
+    <row r="61" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E61" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="62" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F62" t="s">
+    <row r="62" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E62" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="64" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F64" t="s">
+    <row r="64" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E64" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Soulbound and Camille books
</commit_message>
<xml_diff>
--- a/docs/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/docs/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CEE795-1CD7-47F0-AD13-D3A5D5F1ED52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE53BA5-2E0F-4390-A5B6-9DCC7A676FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="345">
   <si>
     <t>Höllisch</t>
   </si>
@@ -390,9 +390,6 @@
     <t>(kein Anagramm)</t>
   </si>
   <si>
-    <t>Avarice in Loss</t>
-  </si>
-  <si>
     <t>Lust</t>
   </si>
   <si>
@@ -456,9 +453,6 @@
     <t>Sorrow out of Death</t>
   </si>
   <si>
-    <t>Anger out of Dread</t>
-  </si>
-  <si>
     <t>Hunger</t>
   </si>
   <si>
@@ -642,9 +636,6 @@
     <t>4/Envy</t>
   </si>
   <si>
-    <t>5/avarice</t>
-  </si>
-  <si>
     <t>6/Sorrow</t>
   </si>
   <si>
@@ -747,12 +738,6 @@
     <t>The first is Ishfotum that reigns in her malice over the children of pride</t>
   </si>
   <si>
-    <t>many Time</t>
-  </si>
-  <si>
-    <t>many few</t>
-  </si>
-  <si>
     <t>Doubt</t>
   </si>
   <si>
@@ -966,15 +951,9 @@
     <t>many many many</t>
   </si>
   <si>
-    <t>Krik-Ref</t>
-  </si>
-  <si>
     <t>Part</t>
   </si>
   <si>
-    <t>To Fey-Erk-Ri Va-Nai-Oor-Kor Krik-Ref Iv-Kar Foy Ru-Kor</t>
-  </si>
-  <si>
     <t>Het-Ay Het-Foy-Shi-Kar To Het-Kor Mirr Esh Tra Ke-Ay-Kor</t>
   </si>
   <si>
@@ -1044,13 +1023,43 @@
     <t>many Body Word</t>
   </si>
   <si>
-    <t>Krik-Ikt-Ike-Tra-Kor</t>
-  </si>
-  <si>
-    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Krik Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
-  </si>
-  <si>
     <t>Movement</t>
+  </si>
+  <si>
+    <t>Anger in Dread</t>
+  </si>
+  <si>
+    <t>Avarice out of Loss</t>
+  </si>
+  <si>
+    <t>fear ending</t>
+  </si>
+  <si>
+    <t>Time Ending</t>
+  </si>
+  <si>
+    <t>Veek-Ref</t>
+  </si>
+  <si>
+    <t>Veek-Ikt-Ike-Tra-Kor</t>
+  </si>
+  <si>
+    <t>To Fey-Erk-Ri Va-Nai-Oor-Kor Veek-Ref Iv-Kar Foy Ru-Kor</t>
+  </si>
+  <si>
+    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
+  </si>
+  <si>
+    <t>5/Avarice</t>
+  </si>
+  <si>
+    <t>Blood</t>
+  </si>
+  <si>
+    <t>Ikt-Ru</t>
+  </si>
+  <si>
+    <t>Soulf o Body</t>
   </si>
 </sst>
 </file>
@@ -1621,10 +1630,10 @@
     </row>
     <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>32</v>
@@ -1657,10 +1666,10 @@
         <v>93</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Q2" s="11" t="s">
         <v>10</v>
@@ -1672,7 +1681,7 @@
         <v>31</v>
       </c>
       <c r="T2" s="11" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="U2" s="12" t="s">
         <v>38</v>
@@ -1680,69 +1689,69 @@
     </row>
     <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>186</v>
-      </c>
       <c r="I3" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q3" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>194</v>
-      </c>
       <c r="R3" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="16"/>
@@ -1764,10 +1773,10 @@
     </row>
     <row r="5" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>39</v>
@@ -1782,7 +1791,7 @@
         <v>13</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J5" s="11" t="s">
         <v>14</v>
@@ -1791,13 +1800,13 @@
         <v>15</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M5" s="11" t="s">
         <v>34</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="O5" s="11" t="s">
         <v>35</v>
@@ -1820,31 +1829,31 @@
     </row>
     <row r="6" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>225</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J6" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>188</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>190</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>91</v>
@@ -1853,33 +1862,33 @@
         <v>34</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E7" s="18"/>
       <c r="F7" s="19"/>
@@ -1900,10 +1909,10 @@
     </row>
     <row r="8" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>16</v>
@@ -1930,7 +1939,7 @@
         <v>104</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>21</v>
@@ -1956,19 +1965,19 @@
     </row>
     <row r="9" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B9" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C9" t="s">
         <v>86</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>94</v>
@@ -1980,37 +1989,37 @@
         <v>72</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="M9" s="6" t="s">
         <v>112</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2066,13 +2075,13 @@
         <v>99</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>79</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2083,42 +2092,42 @@
         <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="I12" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="J12" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="K12" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="L12" s="9" t="s">
         <v>204</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C13" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E13" s="20"/>
       <c r="F13" s="21"/>
@@ -2134,7 +2143,7 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>240</v>
+        <v>336</v>
       </c>
       <c r="C14" t="s">
         <v>95</v>
@@ -2142,13 +2151,13 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B15" t="s">
-        <v>241</v>
+        <v>335</v>
       </c>
       <c r="C15" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E15" t="s">
         <v>40</v>
@@ -2159,30 +2168,30 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B16" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E16" t="s">
         <v>41</v>
       </c>
       <c r="N16" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B17" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C17" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E17" t="s">
         <v>42</v>
@@ -2190,13 +2199,13 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>142</v>
+      </c>
+      <c r="B18" t="s">
+        <v>241</v>
+      </c>
+      <c r="C18" t="s">
         <v>144</v>
-      </c>
-      <c r="B18" t="s">
-        <v>246</v>
-      </c>
-      <c r="C18" t="s">
-        <v>146</v>
       </c>
       <c r="E18" t="s">
         <v>73</v>
@@ -2211,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="V18" t="s">
         <v>114</v>
@@ -2222,10 +2231,10 @@
         <v>92</v>
       </c>
       <c r="B19" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="C19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E19" t="s">
         <v>74</v>
@@ -2240,13 +2249,13 @@
         <v>117</v>
       </c>
       <c r="S19" t="s">
+        <v>137</v>
+      </c>
+      <c r="T19" t="s">
         <v>138</v>
       </c>
-      <c r="T19" t="s">
-        <v>139</v>
-      </c>
       <c r="V19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="W19" t="s">
         <v>120</v>
@@ -2254,13 +2263,13 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B20" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C20" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E20" t="s">
         <v>43</v>
@@ -2272,16 +2281,16 @@
         <v>76</v>
       </c>
       <c r="Q20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="S20" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="T20" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="V20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.3">
@@ -2289,7 +2298,7 @@
         <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C21" t="s">
         <v>97</v>
@@ -2298,33 +2307,33 @@
         <v>44</v>
       </c>
       <c r="N21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O21" t="s">
         <v>77</v>
       </c>
       <c r="Q21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="S21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="T21" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="V21" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>254</v>
+      </c>
+      <c r="B22" t="s">
+        <v>258</v>
+      </c>
+      <c r="C22" t="s">
         <v>259</v>
-      </c>
-      <c r="B22" t="s">
-        <v>263</v>
-      </c>
-      <c r="C22" t="s">
-        <v>264</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
@@ -2339,24 +2348,24 @@
         <v>118</v>
       </c>
       <c r="S22" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="T22" t="s">
+        <v>164</v>
+      </c>
+      <c r="V22" t="s">
         <v>166</v>
-      </c>
-      <c r="V22" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B23" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="C23" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="N23" t="s">
         <v>101</v>
@@ -2365,27 +2374,27 @@
         <v>99</v>
       </c>
       <c r="Q23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="S23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="T23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="V23" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B24" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C24" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="E24" t="s">
         <v>46</v>
@@ -2394,30 +2403,30 @@
         <v>102</v>
       </c>
       <c r="O24" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q24" t="s">
-        <v>121</v>
+        <v>334</v>
       </c>
       <c r="S24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T24" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="V24" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B25" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C25" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
@@ -2429,27 +2438,27 @@
         <v>79</v>
       </c>
       <c r="Q25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="T25" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="V25" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B26" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C26" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="E26" t="s">
         <v>48</v>
@@ -2458,30 +2467,30 @@
         <v>103</v>
       </c>
       <c r="O26" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q26" t="s">
-        <v>143</v>
+        <v>333</v>
       </c>
       <c r="S26" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="T26" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="V26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="B27" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="C27" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E27" t="s">
         <v>49</v>
@@ -2489,13 +2498,13 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="B28" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C28" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="E28" t="s">
         <v>50</v>
@@ -2503,30 +2512,30 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B29" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="C29" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="E29" t="s">
         <v>51</v>
       </c>
       <c r="N29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B30" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="C30" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="E30" t="s">
         <v>52</v>
@@ -2535,35 +2544,35 @@
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B31" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="C31" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
       </c>
       <c r="N31" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B32" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="C32" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="E32" t="s">
         <v>54</v>
@@ -2572,35 +2581,35 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B33" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="C33" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="N33" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B34" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C34" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E34" t="s">
         <v>56</v>
@@ -2609,35 +2618,35 @@
         <v>3</v>
       </c>
       <c r="N34" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B35" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C35" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="E35" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="N35" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B36" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C36" t="s">
-        <v>313</v>
+        <v>337</v>
       </c>
       <c r="E36" t="s">
         <v>57</v>
@@ -2646,69 +2655,69 @@
         <v>4</v>
       </c>
       <c r="N36" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="B37" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="C37" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="E37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N37" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>310</v>
+      </c>
+      <c r="B38" t="s">
+        <v>316</v>
+      </c>
+      <c r="C38" t="s">
         <v>317</v>
-      </c>
-      <c r="B38" t="s">
-        <v>323</v>
-      </c>
-      <c r="C38" t="s">
-        <v>324</v>
       </c>
       <c r="M38">
         <v>5</v>
       </c>
       <c r="N38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="B39" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="C39" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="E39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="B40" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="C40" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E40" t="s">
         <v>59</v>
@@ -2717,32 +2726,32 @@
         <v>6</v>
       </c>
       <c r="N40" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="B41" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="C41" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="N41" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="B42" t="s">
+        <v>331</v>
+      </c>
+      <c r="C42" t="s">
         <v>338</v>
-      </c>
-      <c r="C42" t="s">
-        <v>339</v>
       </c>
       <c r="E42" t="s">
         <v>60</v>
@@ -2751,15 +2760,24 @@
         <v>7</v>
       </c>
       <c r="N42" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>342</v>
+      </c>
+      <c r="B43" t="s">
+        <v>344</v>
+      </c>
+      <c r="C43" t="s">
+        <v>343</v>
+      </c>
       <c r="E43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
@@ -2767,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="N44" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
@@ -2775,7 +2793,7 @@
         <v>62</v>
       </c>
       <c r="N45" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
@@ -2783,7 +2801,7 @@
         <v>63</v>
       </c>
       <c r="N46" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
@@ -2791,7 +2809,7 @@
         <v>64</v>
       </c>
       <c r="N47" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
@@ -2799,7 +2817,7 @@
         <v>65</v>
       </c>
       <c r="N48" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="49" spans="5:14" x14ac:dyDescent="0.3">
@@ -2807,7 +2825,7 @@
         <v>66</v>
       </c>
       <c r="N49" t="s">
-        <v>315</v>
+        <v>339</v>
       </c>
     </row>
     <row r="50" spans="5:14" x14ac:dyDescent="0.3">
@@ -2815,12 +2833,12 @@
         <v>67</v>
       </c>
       <c r="N50" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N51" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
     </row>
     <row r="52" spans="5:14" x14ac:dyDescent="0.3">
@@ -2828,7 +2846,7 @@
         <v>89</v>
       </c>
       <c r="N52" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="53" spans="5:14" x14ac:dyDescent="0.3">
@@ -2844,12 +2862,12 @@
         <v>108</v>
       </c>
       <c r="N54" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="55" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N55" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Camill Buch und Story 10 udpate
</commit_message>
<xml_diff>
--- a/docs/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/docs/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA8F24B-AB5D-4BB1-A540-7888679420E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C7D215-4FF9-4E4D-98AF-82CBC1EDB488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="354">
   <si>
     <t>Höllisch</t>
   </si>
@@ -1056,10 +1056,37 @@
     <t>Ikt-Ru</t>
   </si>
   <si>
-    <t>Soulf o Body</t>
-  </si>
-  <si>
     <t xml:space="preserve">Das Zählsystem ist ein Oktontalsystem von 1-7. </t>
+  </si>
+  <si>
+    <t>Shkarhound</t>
+  </si>
+  <si>
+    <t>Anger Feeder</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Soulf of Body</t>
+  </si>
+  <si>
+    <t>Feeder</t>
+  </si>
+  <si>
+    <t>Fullness filling</t>
+  </si>
+  <si>
+    <t>Raa-Kor</t>
+  </si>
+  <si>
+    <t>Fullness Filler</t>
+  </si>
+  <si>
+    <t>Raa-Esh</t>
+  </si>
+  <si>
+    <t>Kash-Raa-Esh</t>
   </si>
 </sst>
 </file>
@@ -2768,7 +2795,7 @@
         <v>341</v>
       </c>
       <c r="B43" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="C43" t="s">
         <v>342</v>
@@ -2781,6 +2808,15 @@
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>142</v>
+      </c>
+      <c r="B44" t="s">
+        <v>142</v>
+      </c>
+      <c r="C44" t="s">
+        <v>25</v>
+      </c>
       <c r="M44">
         <v>8</v>
       </c>
@@ -2789,6 +2825,15 @@
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>346</v>
+      </c>
+      <c r="B45" t="s">
+        <v>349</v>
+      </c>
+      <c r="C45" t="s">
+        <v>350</v>
+      </c>
       <c r="E45" t="s">
         <v>62</v>
       </c>
@@ -2797,6 +2842,15 @@
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" t="s">
+        <v>351</v>
+      </c>
+      <c r="C46" t="s">
+        <v>352</v>
+      </c>
       <c r="E46" t="s">
         <v>63</v>
       </c>
@@ -2805,6 +2859,15 @@
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>344</v>
+      </c>
+      <c r="B47" t="s">
+        <v>345</v>
+      </c>
+      <c r="C47" t="s">
+        <v>353</v>
+      </c>
       <c r="E47" t="s">
         <v>64</v>
       </c>
@@ -2872,7 +2935,7 @@
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>